<commit_message>
dev:reorganizado a execução da pipeline
</commit_message>
<xml_diff>
--- a/HyperAutomation/resources/planilha_mestra.xlsx
+++ b/HyperAutomation/resources/planilha_mestra.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados extraidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados extraidos'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados extraidos'!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -539,8 +539,6 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>04/08/2026 16:07:02</t>
@@ -588,16 +586,90 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>04/08/2026 16:07:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>/home/sannyer-carvalho/Documentos/Projects/projeto_fani/empresa_portal_fake/HyperAutomation/resources/Documentos_Aprovados/solicitacao_completa_ana_silva.pdf</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Nome, CPF, E-mail, Telefone, Nascimento, Endereco</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PDF invalido ou nao pode ser lido: Stream has ended unexpectedly</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>18/08/2026 10:13:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>/home/sannyer-carvalho/Documentos/Projects/projeto_fani/empresa_portal_fake/HyperAutomation/resources/Documentos_Aprovados/solicitacao_completa_ana_silva.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ana Silva</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>111.222.333-44</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ana.silva@exemplo.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>(92) 98888-1111</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>15/05/1992</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Rua das Palmeiras, 120 - Manaus/AM</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>18/08/2026 10:14:42</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
teste dos processos anteriores
</commit_message>
<xml_diff>
--- a/HyperAutomation/resources/planilha_mestra.xlsx
+++ b/HyperAutomation/resources/planilha_mestra.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados extraidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados extraidos'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados extraidos'!$A$1:$K$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -539,8 +539,6 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>04/08/2026 16:07:02</t>
@@ -588,16 +586,63 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>04/08/2026 16:07:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C:\Users\user\Documents\empresa_portal_fake\HyperAutomation\resources\Documentos_Aprovados\Documento_do_Cliente_02033414221.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fani</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>020.334.142-21</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fani.souza19@gmail.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>(92) 99503-7524</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Rua Rio Purus, 915 - Bairro Taruma-Acu - Manaus/AM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>18/08/2026 10:04:54</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: separa execucao do processo 1 e 2, remove docx temporarios e aprimora validacao multi-arquivos
</commit_message>
<xml_diff>
--- a/HyperAutomation/resources/planilha_mestra.xlsx
+++ b/HyperAutomation/resources/planilha_mestra.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C:\Users\Turma02\Documents\HYPERAUTOMATION\PROJETO FINAL\empresa_portal_fake\HyperAutomation\resources\Documentos_Aprovados\Documentos_do_cliente_03536054250.pdf</t>
+          <t>C:\Users\user\Documents\empresa_portal_fake\HyperAutomation\resources\Documentos_Aprovados\Documentos_do_cliente_03536054250.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -561,6 +561,7 @@
           <t>035.360.542-50</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>(92) 99982-7524</t>
@@ -593,7 +594,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>24/08/2026 17:41:27</t>
+          <t>24/08/2026 21:34:48</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">

</xml_diff>